<commit_message>
Add the Audi MMI 2G limitation to the sheet
Al 7-lea model citit. Text diferit de tiparul BMW: cere AUX activat si mufa
AUX in, si nu merge pe masinile cu Audi CD Changer. Produsul lor e o interfata
CarPlay pentru MMI 2G, deci se compara cu module-carplay, nu cu navigatiile.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -664,30 +664,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -697,49 +697,49 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,63 +749,71 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -817,7 +825,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -826,7 +834,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -853,6 +861,50 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Harvest 17 models from the live site into the Limitări sheet
Ford S-Max si Mondeo IV aduc un tip nou, chiar la nivel de masina: daca masina
nu are plus contact in mufa de alimentare a radioului original, e nevoie de
cablu suplimentar. Restul modelelor citite (Tiguan, Focus II, Scirocco,
Octavia II, Passat B6/B7, Touran, Polo 6R, Viano, Zafira B, Golf 5) nu au
limitari deloc.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -508,30 +508,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bmw seria 1</t>
+          <t>ford s max</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>bmw seria 1 e81 e87</t>
+          <t>ford s max 1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -541,19 +541,19 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina are incalzire in scaune, butoanele se vor reloca, rama avand spatiu pentru acestea in partea inferioara. Vezi detalii aici.</t>
+          <t>Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-seria-1-e81-e87-2003-2013/navigatie-dedicata-cu-android-bmw-seria-1-e81-e87-2007-2013-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-s-max-1-2006-2014/navigatie-dedicata-cu-android-ford-s-max-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -565,25 +565,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bmw seria 3</t>
+          <t>bmw seria 1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>bmw seria 3 e90</t>
+          <t>bmw seria 1 e81 e87</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina are incalzire in scaune, butoanele se vor reloca, rama avand spatiu pentru acestea in partea inferioara. Vezi detalii aici.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -605,37 +605,37 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-seria-3-e90-2004-2013/navigatie-dedicata-cu-android-bmw-seria-3-e90-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-seria-1-e81-e87-2003-2013/navigatie-dedicata-cu-android-bmw-seria-1-e81-e87-2007-2013-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>ford mondeo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -657,37 +657,37 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>bmw seria 3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>bmw seria 3 e90</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -697,49 +697,49 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-seria-3-e90-2004-2013/navigatie-dedicata-cu-android-bmw-seria-3-e90-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,49 +749,49 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -801,105 +801,789 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>cere cablu/adaptor separat</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>bmw</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>bmw x1 e84 cic</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2009-2015</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>bmw x1 e84</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2009-2015</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>vw tiguan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2007-2016</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>vw tiguan 1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2007-2018</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ford focus</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>51</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>42</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>vw scirocco</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2008-2018</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>42</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>vw scirocco</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2008-2018</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>skoda</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>skoda octavia</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2004-2013</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>33</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>skoda octavia 2</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2004-2013</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>vw passat b6</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2005-2010</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>33</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>vw passat b6 b7</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2005-2015</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>vw polo 6r</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2009-2018</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>33</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>vw polo 6r</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2009-2018</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>vw touran</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2003-2013</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>33</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>vw touran 1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>opel</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>opel zafira</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2005-2014</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>26</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>opel zafira b</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2005-2014</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>vw passat b7</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2010-2014</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>25</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>vw passat b6 b7</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2005-2015</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>mercedes benz viano</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2003-2014</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>24</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>mercedes viano</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2003-2014</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>12</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>mercedes viano</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2003-2014</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>9</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
         <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>

</xml_diff>

<commit_message>
Harvest 20 models: Toyota Corolla E18 brings the clearest car-level limits yet
Corolla E18: nu se monteaza pe masinile cu butonul de avarii PATRAT, si cere
decuparea unei portiuni de plastic din bord — astea sunt ale masinii, nu ale
produsului. Plus cablu adaptor daca are amplificator sau navigatie originala
cu camera.

Fara limitari: Vito, Seat Leon 1P, Viano, Zafira B, Octavia II, Passat B6/B7,
Touran, Polo 6R, Tiguan, Focus II, Scirocco, Golf 5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -976,74 +976,78 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2007-2016</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1057,37 +1061,37 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1101,7 +1105,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
@@ -1113,12 +1117,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1126,12 +1130,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1145,37 +1149,37 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1189,24 +1193,24 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1214,12 +1218,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1233,7 +1237,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -1245,12 +1249,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1258,12 +1262,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1277,7 +1281,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1293,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1302,12 +1306,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1321,37 +1325,37 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1365,37 +1369,37 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1409,37 +1413,37 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1453,37 +1457,37 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1497,37 +1501,37 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1541,37 +1545,37 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1585,6 +1589,226 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>seat</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>seat leon</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2005-2013</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>24</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>seat leon 1p</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2005-2013</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>12</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>mercedes viano</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2003-2014</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>12</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>mercedes vito</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>dupa 2003</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>10</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>9</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest up to 22 models (Fiat 500, Ford Fiesta V — both without limits)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1508,17 +1508,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1545,24 +1545,24 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1570,12 +1570,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1589,24 +1589,24 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1614,12 +1614,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1633,7 +1633,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1645,25 +1645,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1677,37 +1677,37 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1721,37 +1721,37 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1765,37 +1765,37 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1809,6 +1809,138 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>10</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>9</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 25 models: Toyota confirms a real per-car pattern
RAV4 IV repeta tiparul de la Corolla E18 (cablu adaptor daca are amplificator
sau navigatie originala + camera). BMW X3 F25, tot interfata: cere AUX activat,
iar la masinile cu camere 360 din fabrica nu se mai poate schimba modul de
vizualizare. Auris E15 fara limitari.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -716,30 +716,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4 4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,49 +749,49 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-rav4-4-2013-2018/navigatie-dedicata-cu-android-toyota-rav4-iv-2013-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -801,49 +801,49 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -853,49 +853,49 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,49 +905,49 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -969,33 +969,37 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>honda crv</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1005,225 +1009,253 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2008-2018</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1237,37 +1269,37 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1281,7 +1313,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
@@ -1293,25 +1325,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1325,7 +1357,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1337,25 +1369,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1369,37 +1401,37 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1413,37 +1445,37 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1457,7 +1489,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1469,25 +1501,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1501,37 +1533,37 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1545,37 +1577,37 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1589,37 +1621,37 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1633,37 +1665,37 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1677,24 +1709,24 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1702,12 +1734,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1721,37 +1753,37 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1765,7 +1797,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1777,25 +1809,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1809,37 +1841,37 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1853,37 +1885,37 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1897,37 +1929,37 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1941,6 +1973,226 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>12</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>mercedes viano</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2003-2014</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>12</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>mercedes vito</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>dupa 2003</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>10</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>9</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 28 models: Ford Kuga I needs an A/C module with factory Blaupunkt
Kuga I e cea mai specifica de pana acum: cu navigatie originala Blaupunkt
cere un modul de control aer conditionat, vandut separat. Ei au o categorie
intreaga /cabluri-si-canbus-uri/ — exact accesoriile pe care noi nu le avem.
Honda CR-V III repeta formula cu navigatia de fabrica.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -872,30 +872,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga 1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -917,24 +917,24 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -942,12 +942,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -957,49 +957,49 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1009,49 +1009,49 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1073,37 +1073,37 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1113,19 +1113,19 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1137,12 +1137,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1165,45 +1165,49 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>bmw x3 f25 cic</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2011-2017</t>
+        </is>
+      </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1213,107 +1217,119 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ford focus</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2004-2011</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1325,25 +1341,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1357,37 +1373,37 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1401,37 +1417,37 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1445,7 +1461,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1457,25 +1473,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1489,24 +1505,24 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1514,12 +1530,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1533,7 +1549,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -1545,12 +1561,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1558,12 +1574,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1577,37 +1593,37 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1621,37 +1637,37 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1665,37 +1681,37 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1709,37 +1725,37 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1753,37 +1769,37 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1797,24 +1813,24 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1822,12 +1838,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1841,24 +1857,24 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1866,12 +1882,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1885,24 +1901,24 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1910,12 +1926,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1929,37 +1945,37 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1973,37 +1989,37 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2017,37 +2033,37 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2061,37 +2077,37 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2105,37 +2121,37 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2149,37 +2165,37 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2193,6 +2209,138 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>9</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>9</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 30 models: Ford Focus III loses acoustic parking sensors
Focus III: cu 12 senzori de parcare originali, navigatia ii preia doar vizual,
nu si acustic — limitare de functionalitate, nu de montaj. Transit fara.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -820,30 +820,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -865,24 +865,24 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ford kuga</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -890,12 +890,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ford kuga 1</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -917,37 +917,37 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga 1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -969,24 +969,24 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -994,12 +994,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1009,49 +1009,49 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>honda cr v 3</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1113,49 +1113,49 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1165,49 +1165,49 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1229,7 +1229,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1241,12 +1241,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1269,45 +1269,49 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>bmw x3 f25 cic</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2011-2017</t>
+        </is>
+      </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1317,107 +1321,119 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ford focus</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2004-2011</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1429,25 +1445,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1461,37 +1477,37 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1505,37 +1521,37 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1549,7 +1565,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1561,25 +1577,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1593,24 +1609,24 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1618,12 +1634,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1637,7 +1653,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1665,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1662,12 +1678,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1681,37 +1697,37 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1725,37 +1741,37 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1769,37 +1785,37 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1813,37 +1829,37 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1857,37 +1873,37 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1901,24 +1917,24 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1926,12 +1942,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1945,24 +1961,24 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1970,12 +1986,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1989,24 +2005,24 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2014,12 +2030,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2033,37 +2049,37 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2077,37 +2093,37 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2121,37 +2137,37 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2165,7 +2181,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2177,25 +2193,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2209,37 +2225,37 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2253,37 +2269,37 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2297,37 +2313,37 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2341,6 +2357,182 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>9</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ford transit connect</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2008-2011</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>9</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>9</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 35 models: Opel Astra H drops the climate display
Astra H: clima ramane pe butoanele fizice, dar informatiile nu mai apar pe
ecran. Galaxy II repeta plus-contactul de la S-Max. Ford Ranger are varianta
dedicata 'cu navigatie originala' si zero limitari — inca un semn ca
restrictia cu navigatia de fabrica e a produsului lor, nu a masinii.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -664,30 +664,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bmw seria 3</t>
+          <t>ford galaxy 2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>bmw seria 3 e90</t>
+          <t>ford galaxy 2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -697,49 +697,49 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-seria-3-e90-2004-2013/navigatie-dedicata-cu-android-bmw-seria-3-e90-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-galaxy-2-2006-2015/navigatie-dedicata-cu-android-ford-galaxy-2008-2015-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>toyota rav4</t>
+          <t>bmw seria 3</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>toyota rav4 4</t>
+          <t>bmw seria 3 e90</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,49 +749,49 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-rav4-4-2013-2018/navigatie-dedicata-cu-android-toyota-rav4-iv-2013-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-seria-3-e90-2004-2013/navigatie-dedicata-cu-android-bmw-seria-3-e90-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4 4</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -801,49 +801,49 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-rav4-4-2013-2018/navigatie-dedicata-cu-android-toyota-rav4-iv-2013-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -853,49 +853,49 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -917,37 +917,37 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ford kuga</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2004-2010</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ford kuga 1</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -957,49 +957,49 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
+          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>afisaj/comenzi clima</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1021,7 +1021,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
@@ -1033,25 +1033,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>ford kuga</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>ford kuga 1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1061,49 +1061,49 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>honda cr v 3</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1113,49 +1113,49 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1165,49 +1165,49 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1217,49 +1217,49 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1269,49 +1269,49 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1333,7 +1333,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1358,12 +1358,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,45 +1373,49 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>bmw x3 f25 cic</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2011-2017</t>
+        </is>
+      </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1421,107 +1425,119 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ford focus</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2004-2011</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1533,25 +1549,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1565,37 +1581,37 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1609,37 +1625,37 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1653,7 +1669,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1665,25 +1681,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1697,24 +1713,24 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1722,12 +1738,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1741,7 +1757,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1769,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1766,12 +1782,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1785,37 +1801,37 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1829,37 +1845,37 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1873,7 +1889,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1885,25 +1901,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1917,37 +1933,37 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1961,37 +1977,37 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2005,37 +2021,37 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2049,37 +2065,37 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2093,24 +2109,24 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2118,12 +2134,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2137,37 +2153,37 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2181,37 +2197,37 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2225,7 +2241,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2237,25 +2253,25 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2269,37 +2285,37 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2313,37 +2329,37 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2357,37 +2373,37 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2401,37 +2417,37 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2445,37 +2461,37 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2489,37 +2505,37 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2533,6 +2549,226 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>9</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ford transit connect</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2008-2011</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>renault</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>renault megane iii</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>9</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>renault megane 3</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>9</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>9</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 38 models: Hyundai ix35 repeats the Toyota amplifier/camera pattern
Dacia Duster I, Logan II si Renault Megane III — fara limitari.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1288,30 +1288,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>hyundai</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,49 +1321,49 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,19 +1373,19 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1397,12 +1397,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1410,12 +1410,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1496,26 +1496,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>bmw x3 f25 nbt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2011-2017</t>
+        </is>
+      </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1525,93 +1529,97 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>2007-2016</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1625,37 +1633,37 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1669,7 +1677,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
@@ -1681,12 +1689,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1694,12 +1702,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1713,37 +1721,37 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1757,24 +1765,24 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>vw jetta</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2006-2010</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1782,12 +1790,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>vw jetta 3</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1801,7 +1809,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -1813,12 +1821,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1826,12 +1834,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1845,7 +1853,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1865,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1870,12 +1878,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1889,7 +1897,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1909,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1914,12 +1922,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1933,37 +1941,37 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2015-2022</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1977,24 +1985,24 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2002,12 +2010,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2021,37 +2029,37 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2065,37 +2073,37 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2109,37 +2117,37 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2153,24 +2161,24 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2178,12 +2186,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2197,24 +2205,24 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2222,12 +2230,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2241,7 +2249,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2253,12 +2261,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2266,12 +2274,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2285,24 +2293,24 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2310,12 +2318,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2329,37 +2337,37 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2373,37 +2381,37 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2417,37 +2425,37 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2461,37 +2469,37 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2505,7 +2513,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2517,25 +2525,25 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2549,37 +2557,37 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2015-2020</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2593,37 +2601,37 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2637,37 +2645,37 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>renault megane iii</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>renault megane 3</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2681,37 +2689,37 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2725,24 +2733,24 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>fiat 500 l</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2750,12 +2758,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2769,7 +2777,227 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ford transit connect</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2008-2011</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>9</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>renault</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>renault megane iii</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>renault megane 3</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>9</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>9</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>dacia logan</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>dacia logan 2</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harvest 40 models; the limitations fall into 6 recurring patterns
Kia Sportage III si Nissan Qashqai I confirma tiparul cu cablul adaptor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1340,30 +1340,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>kia sportage 3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,49 +1373,49 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1449,12 +1449,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1462,12 +1462,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1477,19 +1477,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1548,26 +1548,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>bmw x3 f25 nbt</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2011-2017</t>
+        </is>
+      </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1577,107 +1581,115 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>NISSAN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>2007-2016</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>nissan qashqai 1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>cere cablu/adaptor separat</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ford focus</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>2004-2011</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1689,25 +1701,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1721,37 +1733,37 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1765,37 +1777,37 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1809,7 +1821,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1821,25 +1833,25 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>vw jetta</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2006-2010</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>vw jetta 3</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1853,24 +1865,24 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1878,12 +1890,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1897,7 +1909,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -1909,12 +1921,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1922,12 +1934,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1941,7 +1953,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1953,12 +1965,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1966,12 +1978,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1985,37 +1997,37 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2015-2022</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2029,37 +2041,37 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2073,37 +2085,37 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2117,37 +2129,37 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2161,37 +2173,37 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2205,37 +2217,37 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2249,24 +2261,24 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2274,12 +2286,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2293,24 +2305,24 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2318,12 +2330,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2337,24 +2349,24 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2362,12 +2374,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2381,37 +2393,37 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2010-2013</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2425,37 +2437,37 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2469,24 +2481,24 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2494,12 +2506,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2513,37 +2525,37 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2557,37 +2569,37 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2015-2020</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2601,37 +2613,37 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2645,24 +2657,24 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2015-2020</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2670,12 +2682,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2689,37 +2701,37 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2733,37 +2745,37 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2777,7 +2789,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2789,25 +2801,25 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2821,24 +2833,24 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>renault megane iii</t>
+          <t>fiat 500 l</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2846,12 +2858,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>renault megane 3</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2865,24 +2877,24 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>ford transit connect</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2890,12 +2902,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2909,24 +2921,24 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>renault</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>renault megane iii</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2934,12 +2946,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>renault megane 3</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2953,37 +2965,37 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>dacia logan</t>
+          <t>toyota corolla e15</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2007-2013</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>toyota corolla e15</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2007-2013</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2997,6 +3009,94 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>9</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>dacia logan</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>dacia logan 2</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 47 models using the sitemap shortcut
Ford Transit dupa 2014: daca masina are ecran pe bord cu data si ora, ramane
un spatiu gol in spatele navigatiei dupa montaj.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1184,17 +1184,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>dupa 2021</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1202,12 +1202,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>honda cr v 3</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1217,36 +1217,36 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford transit connect</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>dupa 2013</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1269,36 +1269,36 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>hyundai</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,36 +1321,36 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>kia sportage</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1358,12 +1358,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>kia sportage 3</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,49 +1373,49 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>hyundai</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1425,49 +1425,49 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>kia sportage 3</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1477,49 +1477,49 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2014-2020</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1541,37 +1541,37 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1593,33 +1593,37 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NISSAN</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>ford transit courier</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2014-2018</t>
+        </is>
+      </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>nissan qashqai 1</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1629,45 +1633,49 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>bmw x1 e84 cic</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2009-2015</t>
+        </is>
+      </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1677,7 +1685,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1689,213 +1697,237 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>NISSAN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>2004-2008</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>nissan qashqai 1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>cere cablu/adaptor separat</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2008-2018</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1909,32 +1941,32 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>vw jetta</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2006-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>vw jetta 3</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1953,7 +1985,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
@@ -1965,25 +1997,25 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1997,7 +2029,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2009,25 +2041,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2041,24 +2073,24 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2066,12 +2098,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2085,37 +2117,37 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2015-2022</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2129,37 +2161,37 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2173,37 +2205,37 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2217,7 +2249,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2229,25 +2261,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2261,37 +2293,37 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2305,37 +2337,37 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2349,37 +2381,37 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2393,37 +2425,37 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2437,24 +2469,24 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2462,12 +2494,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2481,37 +2513,37 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2010-2013</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2525,37 +2557,37 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2569,37 +2601,37 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2613,37 +2645,37 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2657,37 +2689,37 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2015-2020</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2701,37 +2733,37 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2745,37 +2777,37 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2789,37 +2821,37 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2833,37 +2865,37 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2877,37 +2909,37 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2921,37 +2953,37 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>renault megane iii</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>renault megane 3</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2965,37 +2997,37 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3009,37 +3041,37 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3053,7 +3085,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3097,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>dacia logan</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3074,7 +3106,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -3101,6 +3133,710 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>toyota auris e15</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2006-2012</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>18</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>toyota auris e15</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2006-2012</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2005-2014</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>15</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>vw multivan t5</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2003-2009</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>15</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>vw multivan t5</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2003-2015</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>vw transporter t5</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2003-2009</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>15</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>vw transporter t5</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2003-2015</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>dacia duster</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2015-2020</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>12</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>dacia duster 1</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2010-2018</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>12</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>mercedes viano</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2003-2014</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>12</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>mercedes vito</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>dupa 2003</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>9</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ford transit connect</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2008-2011</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>9</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>renault</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>renault megane iii</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>9</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>renault megane 3</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>skoda</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2017-2019</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>9</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2011-2019</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>9</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>9</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>9</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>vw golf plus</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2004-2014</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>dacia logan</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>3</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>dacia logan 2</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Harvest 51 models: two new physical/audio limitations
VW Transporter T6: rotile de reglare de sub grilele de ventilatie trebuie
scoase ca sa intre navigatia. Mitsubishi ASX: amplificator Rockford cere
cablu adaptor separat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -768,30 +768,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>toyota rav4</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2015-2019</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>toyota rav4 4</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -801,49 +801,49 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-rav4-4-2013-2018/navigatie-dedicata-cu-android-toyota-rav4-iv-2013-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4 4</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -853,49 +853,49 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-rav4-4-2013-2018/navigatie-dedicata-cu-android-toyota-rav4-iv-2013-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,36 +905,36 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2004-2010</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -942,12 +942,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -957,49 +957,49 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>afisaj/comenzi clima</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2004-2010</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1009,36 +1009,36 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>afisaj/comenzi clima</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ford kuga</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1046,12 +1046,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ford kuga 1</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1073,37 +1073,37 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga 1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1125,24 +1125,24 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1165,19 +1165,19 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
@@ -1189,25 +1189,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>dupa 2021</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1217,19 +1217,19 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1241,12 +1241,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>dupa 2013</t>
+          <t>dupa 2021</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1288,17 +1288,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford transit connect</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>dupa 2013</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>honda cr v 3</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,19 +1321,19 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1358,12 +1358,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,36 +1373,36 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>hyundai</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1410,12 +1410,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1425,36 +1425,36 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>hyundai</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>kia sportage</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1462,12 +1462,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>kia sportage 3</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1489,37 +1489,37 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2014-2020</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>kia sportage 3</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1529,49 +1529,49 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1581,19 +1581,19 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
@@ -1605,16 +1605,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ford transit courier</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2014-2018</t>
+          <t>2014-2020</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1652,30 +1652,30 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2017-2019</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1685,49 +1685,49 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2020-2022</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1737,49 +1737,49 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2019-2024</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1801,33 +1801,37 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NISSAN</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>ford focus 3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2011-2019</t>
+        </is>
+      </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>nissan qashqai 1</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1837,45 +1841,49 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>ford transit courier</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2014-2018</t>
+        </is>
+      </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1885,239 +1893,271 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>NISSAN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>2008-2018</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>nissan qashqai 1</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>cere cablu/adaptor separat</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>2004-2013</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2129,25 +2169,25 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>vw jetta</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2006-2010</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>vw jetta 3</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2161,37 +2201,37 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2205,7 +2245,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
@@ -2217,25 +2257,25 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2249,7 +2289,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2261,25 +2301,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2293,37 +2333,37 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2015-2022</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2337,37 +2377,37 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2381,37 +2421,37 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2425,7 +2465,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2437,25 +2477,25 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2469,37 +2509,37 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2513,37 +2553,37 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>vw touran 2</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2557,37 +2597,37 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-2-2010-2015/navigatie-dedicata-cu-android-vw-touran-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2601,7 +2641,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
@@ -2613,16 +2653,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2652,30 +2692,30 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2689,37 +2729,37 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2733,24 +2773,24 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2758,12 +2798,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2777,24 +2817,24 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2802,12 +2842,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2821,24 +2861,24 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2846,12 +2886,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2865,24 +2905,24 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2012-2017</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2890,12 +2930,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2909,24 +2949,24 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2934,12 +2974,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2953,24 +2993,24 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2978,12 +3018,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2997,24 +3037,24 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3022,12 +3062,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3041,37 +3081,37 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2010-2013</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3085,37 +3125,37 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3129,37 +3169,37 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3173,19 +3213,19 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3194,16 +3234,16 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3217,7 +3257,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -3234,11 +3274,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3278,11 +3318,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3322,11 +3362,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2015-2020</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -3356,30 +3396,30 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3393,37 +3433,37 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>ford ranger f250</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3437,37 +3477,37 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3481,37 +3521,37 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3525,37 +3565,37 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3569,37 +3609,37 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>renault megane iii</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>renault megane 3</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3613,37 +3653,37 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2011-2016</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3657,37 +3697,37 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2015-2020</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3701,37 +3741,37 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3745,37 +3785,37 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3789,37 +3829,37 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>dacia logan</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3833,6 +3873,358 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>9</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ford transit connect</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2008-2011</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>9</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>renault</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>renault megane iii</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>9</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>renault megane 3</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>skoda</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2017-2019</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>9</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2011-2019</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>9</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>9</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>9</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>vw golf plus</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2004-2014</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>dacia logan</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>3</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>dacia logan 2</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 57 models: Opel Insignia blocked by factory Infinity audio
Insignia A: nu se monteaza pe masinile cu sistem de sunet Infinity din fabrica.
Mazda 3 mentioneaza explicit ca E compatibila cu Bose — util de stiut ca
sistemul audio nu e automat un blocaj.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -976,17 +976,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>kia sorento</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2004-2010</t>
+          <t>2013-2015</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -994,12 +994,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>kia sorento 2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1009,49 +1009,49 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>afisaj/comenzi clima</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>mazda</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2013-2019</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1061,49 +1061,49 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ford kuga</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2004-2010</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ford kuga 1</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1113,49 +1113,49 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
+          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>afisaj/comenzi clima</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1165,49 +1165,49 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1217,19 +1217,19 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
@@ -1241,25 +1241,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford kuga</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>dupa 2021</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford kuga 1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1281,37 +1281,37 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>dupa 2013</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1333,37 +1333,37 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>honda cr v 3</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1385,24 +1385,24 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>dupa 2021</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1410,12 +1410,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1425,36 +1425,36 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>hyundai</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>ford transit connect</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2013</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1462,12 +1462,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1477,36 +1477,36 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>kia sportage</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1514,12 +1514,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>kia sportage 3</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1529,36 +1529,36 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>mitsubishi</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>dupa 2010</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1581,49 +1581,49 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>hyundai</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2014-2020</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1633,49 +1633,49 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>mitsubishi</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>kia sportage 3</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dupa 2010</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1697,7 +1697,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -1714,11 +1714,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1756,30 +1756,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>opel insignia</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2019-2024</t>
+          <t>2008-2013</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>opel insignia a</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2008-2017</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
+          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1801,37 +1801,37 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>opel insignia</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2013-2017</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>opel insignia a</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2008-2017</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1853,7 +1853,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -1865,16 +1865,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ford transit courier</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2014-2018</t>
+          <t>2014-2020</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1912,25 +1912,25 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>kia sorento</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2009-2012</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>kia sorento 2</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1957,37 +1957,37 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>mazda</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>mazda cx 3</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2014-2021</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2013-2019</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1997,49 +1997,49 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2017-2019</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2049,45 +2049,49 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>NISSAN</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>mitsubishi asx</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2020-2022</t>
+        </is>
+      </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>nissan qashqai 1</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2097,45 +2101,49 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
+          <t>toyota avensis</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2015-2018</t>
+        </is>
+      </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2145,19 +2153,19 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2169,39 +2177,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2019-2024</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
@@ -2213,303 +2229,351 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford transit courier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2014-2018</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>vw jetta</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2006-2010</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>vw jetta 3</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>NISSAN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>2005-2010</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>nissan qashqai 1</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>cere cablu/adaptor separat</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>2009-2018</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2521,25 +2585,25 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2553,37 +2617,37 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>vw touran 2</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2597,37 +2661,37 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-2-2010-2015/navigatie-dedicata-cu-android-vw-touran-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2015-2022</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2641,37 +2705,37 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2685,37 +2749,37 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2729,7 +2793,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -2741,25 +2805,25 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2773,37 +2837,37 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2817,37 +2881,37 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2861,37 +2925,37 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2905,37 +2969,37 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw touran 2</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2949,37 +3013,37 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-2-2010-2015/navigatie-dedicata-cu-android-vw-touran-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>vw polo</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2001-2009</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>vw polo 9n</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2001-2012</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2993,37 +3057,37 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-9n-2001-2012/navigatie-dedicata-cu-android-vw-polo-9n-2001-2012-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3037,37 +3101,37 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3081,37 +3145,37 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3125,37 +3189,37 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3169,24 +3233,24 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2012-2017</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3194,12 +3258,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3213,24 +3277,24 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3238,12 +3302,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3257,24 +3321,24 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3282,12 +3346,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3301,24 +3365,24 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3326,12 +3390,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3345,37 +3409,37 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2010-2013</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3389,37 +3453,37 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3433,37 +3497,37 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ford ranger f250</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3477,37 +3541,37 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3521,37 +3585,37 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3565,37 +3629,37 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3609,7 +3673,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -3621,25 +3685,25 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3653,37 +3717,37 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2011-2016</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3697,37 +3761,37 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2015-2020</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3741,37 +3805,37 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3785,37 +3849,37 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3829,37 +3893,37 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3873,37 +3937,37 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>ford ranger f250</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3917,37 +3981,37 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3961,37 +4025,37 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>renault megane iii</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>renault megane 3</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4005,37 +4069,37 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -4049,37 +4113,37 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -4093,37 +4157,37 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2011-2016</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4137,37 +4201,37 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2015-2020</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4181,37 +4245,37 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>dacia logan</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4225,6 +4289,490 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>12</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>mercedes vito</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>dupa 2003</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>10</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>dacia logan 1</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>9</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>dacia logan 1</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2004-2013</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>9</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ford transit connect</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2008-2011</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>9</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>renault</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>renault megane iii</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>9</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>renault megane 3</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>skoda</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2017-2019</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>9</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2011-2019</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>9</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>9</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>9</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>vw golf plus</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2004-2014</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>dacia logan</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>3</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>dacia logan 2</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 62 models: Mercedes W203 needs a 6m fibre-optic cable
W203: sistem audio pe fibra optica (amplificator sau magazie CD) cere un
cablu suplimentar de 6m. Citroen C4 Aircross repeta amplificatorul Rockford
de la Mitsubishi ASX — sunt aceeasi platforma.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -976,17 +976,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>kia sorento</t>
+          <t>ford mondeo 3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2013-2015</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -994,12 +994,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>kia sorento 2</t>
+          <t>ford mondeo 3</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1021,24 +1021,24 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-3-2000-2007/navigatie-dedicata-cu-android-ford-mondeo-iii-2000-2007-clima-automata-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>mazda</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>mazda 3</t>
+          <t>kia sorento</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2013-2015</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1046,12 +1046,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>mazda 3</t>
+          <t>kia sorento 2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2013-2019</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1061,36 +1061,36 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>mazda</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2004-2010</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2013-2019</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1113,36 +1113,36 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>afisaj/comenzi clima</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>toyota avensis t27</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2004-2010</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>toyota avensis t27</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1165,49 +1165,49 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>afisaj/comenzi clima</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1217,36 +1217,36 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ford kuga</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ford kuga 1</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1281,37 +1281,37 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga 1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1333,24 +1333,24 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1358,12 +1358,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,19 +1373,19 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
@@ -1397,25 +1397,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>dupa 2021</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1425,36 +1425,36 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>citroen</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>citroen c4 aircross</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>dupa 2013</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1462,12 +1462,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>citroen c4 aircross</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1477,36 +1477,36 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-aircross-2012-2017/navigatie-dedicata-cu-android-citroen-c4-aircross-2012-2017-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>citroen</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1514,12 +1514,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>honda cr v 3</t>
+          <t>citroen c4 aircross</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1529,36 +1529,36 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-aircross-2012-2017/navigatie-dedicata-cu-android-citroen-c4-aircross-2012-2017-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>dupa 2021</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1581,36 +1581,36 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>hyundai</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>ford transit connect</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2013</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1618,12 +1618,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1633,36 +1633,36 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>kia sportage</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>kia sportage 3</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1685,36 +1685,36 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>mitsubishi</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1722,12 +1722,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>dupa 2010</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1737,36 +1737,36 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>hyundai</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>opel insignia</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2008-2013</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>opel insignia a</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2008-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1789,36 +1789,36 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>opel insignia</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2013-2017</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>opel insignia a</t>
+          <t>kia sportage 3</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2008-2017</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1841,49 +1841,49 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2014-2020</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1893,49 +1893,49 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>kia sorento</t>
+          <t>opel insignia</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2009-2012</t>
+          <t>2008-2013</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>kia sorento 2</t>
+          <t>opel insignia a</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2008-2017</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1945,49 +1945,49 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>mazda</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>mazda cx 3</t>
+          <t>opel insignia</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2014-2021</t>
+          <t>2013-2017</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>mazda 3</t>
+          <t>opel insignia a</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2013-2019</t>
+          <t>2008-2017</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1997,49 +1997,49 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
+          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mitsubishi</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>mercedes benz c class w203</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2000-2004</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>mercedes c class w203</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>dupa 2010</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2049,49 +2049,49 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are sistemul audio pe fibra optica (are amplificator sau magazie de cd-uri) este necesar un cablu suplimentar de 6m care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-c-class-w203-2000-2007/navigatie-dedicata-cu-android-mercedes-c-class-w203-2000-2004-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>mitsubishi</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>mercedes benz c class w203</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2004-2007</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>mercedes c class w203</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dupa 2010</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2101,36 +2101,36 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are sistemul audio pe fibra optica (are amplificator sau magazie de cd-uri) este necesar un cablu suplimentar de 6m care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-c-class-w203-2000-2007/navigatie-dedicata-cu-android-mercedes-c-class-w203-2000-2004-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>toyota avensis</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2015-2018</t>
+          <t>2014-2020</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2138,12 +2138,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>toyota avensis t27</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2153,36 +2153,36 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>kia sorento</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2019-2024</t>
+          <t>2009-2012</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2190,12 +2190,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>kia sorento 2</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2205,49 +2205,49 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2016-2018</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>kia sportage 4</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2016-2021</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2257,49 +2257,49 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-4-2016-2021/navigatie-dedicata-cu-android-kia-sportage-2016-2018-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ford transit courier</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2014-2018</t>
+          <t>2018-2019</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>kia sportage 4</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2016-2021</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2309,49 +2309,49 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-4-2016-2021/navigatie-dedicata-cu-android-kia-sportage-2016-2018-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2019-2021</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>kia sportage 4</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2016-2021</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2361,49 +2361,49 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-4-2016-2021/navigatie-dedicata-cu-android-kia-sportage-2016-2018-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>mazda</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>mazda cx 3</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2014-2021</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2013-2019</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2413,49 +2413,49 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2017-2019</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2465,45 +2465,49 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NISSAN</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
+          <t>mitsubishi asx</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2020-2022</t>
+        </is>
+      </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>nissan qashqai 1</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2513,45 +2517,49 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
+          <t>toyota avensis</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2015-2018</t>
+        </is>
+      </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2561,19 +2569,19 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2585,39 +2593,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2007-2016</t>
+          <t>2019-2024</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
@@ -2629,347 +2645,403 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>ford mondeo</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford mondeo 3</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-3-2000-2007/navigatie-dedicata-cu-android-ford-mondeo-iii-2000-2007-clima-automata-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford transit courier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2014-2018</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr"/>
-      <c r="I45" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>vw jetta</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2006-2010</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>vw jetta 3</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>bmw x3 f25 nbt</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>altceva — de citit</t>
+        </is>
+      </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>NISSAN</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>2009-2018</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>nissan qashqai 1</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr"/>
-      <c r="I49" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>cere cablu/adaptor separat</t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>vw touran</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>2003-2013</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2981,25 +3053,25 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>vw touran 2</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3013,37 +3085,37 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-2-2010-2015/navigatie-dedicata-cu-android-vw-touran-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>vw polo</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2001-2009</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>vw polo 9n</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2001-2012</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3057,37 +3129,37 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-9n-2001-2012/navigatie-dedicata-cu-android-vw-polo-9n-2001-2012-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2015-2022</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3101,37 +3173,37 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3145,37 +3217,37 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3189,7 +3261,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -3201,25 +3273,25 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3233,37 +3305,37 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3277,37 +3349,37 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3321,37 +3393,37 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3365,37 +3437,37 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>vw touran 2</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3409,37 +3481,37 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-2-2010-2015/navigatie-dedicata-cu-android-vw-touran-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>vw polo</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2001-2009</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>vw polo 9n</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2001-2012</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3453,37 +3525,37 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-9n-2001-2012/navigatie-dedicata-cu-android-vw-polo-9n-2001-2012-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3497,37 +3569,37 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3541,37 +3613,37 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3585,37 +3657,37 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3629,24 +3701,24 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2012-2017</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3654,12 +3726,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3673,24 +3745,24 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3698,12 +3770,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3717,24 +3789,24 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3742,12 +3814,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3761,24 +3833,24 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3786,12 +3858,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3805,37 +3877,37 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2010-2013</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3849,37 +3921,37 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3893,37 +3965,37 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3937,37 +4009,37 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ford ranger f250</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3981,37 +4053,37 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4025,37 +4097,37 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4069,7 +4141,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -4081,25 +4153,25 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -4113,7 +4185,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -4125,20 +4197,20 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4157,37 +4229,37 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2011-2016</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4201,7 +4273,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
@@ -4218,11 +4290,11 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2015-2020</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -4252,30 +4324,30 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4289,37 +4361,37 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4333,7 +4405,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -4345,25 +4417,25 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford ranger f250</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4377,37 +4449,37 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4421,37 +4493,37 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4465,37 +4537,37 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4509,37 +4581,37 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>renault megane iii</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>renault megane 3</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4553,37 +4625,37 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>citroen</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4597,37 +4669,37 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-2009-2018/navigatie-dedicata-cu-android-citroen-c4-ii-2009-2018-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-10</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>citroen</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>citroen c4 aircross</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4641,37 +4713,37 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-2009-2018/navigatie-dedicata-cu-android-citroen-c4-ii-2009-2018-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-10</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2011-2016</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4685,37 +4757,37 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2015-2020</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4729,37 +4801,37 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>dacia logan</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4773,6 +4845,490 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>mercedes benz vito viano w639</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2010-2015</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>12</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>mercedes vito</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>dupa 2003</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>10</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>ford focus 2</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2004-2011</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>dacia logan 1</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>9</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>dacia logan 1</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2004-2013</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>fiat</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>fiat 500 l</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>dupa 2012</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>9</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>fiat 500</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2007-2020</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ford</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ford transit connect</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2008-2011</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>9</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>ford transit</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2006-2014</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>renault</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>renault megane iii</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>9</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>renault megane 3</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2009-2016</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>skoda</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2017-2019</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>9</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2011-2019</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>9</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr"/>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>9</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>9</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>vw golf plus</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2004-2014</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>dacia logan</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>3</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>dacia logan 2</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Harvest 67 models: Skoda Superb II blocked by the factory Sound System amp
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/limitari-decizie.xlsx
+++ b/backend/scripts/limitari-decizie.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -768,17 +768,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>skoda superb 2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2015-2019</t>
+          <t>2008-2015</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -786,12 +786,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>skoda superb 2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2008-2015</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -801,49 +801,49 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
+          <t>Nu se poate monta pe masini care au sistem de sunet cu amplificator Sound System.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-superb-2-2008-2015/navigatie-dedicata-cu-android-skoda-superb-ii-2008-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>toyota rav4</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2015-2019</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>toyota rav4 4</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -853,49 +853,49 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-rav4-4-2013-2018/navigatie-dedicata-cu-android-toyota-rav4-iv-2013-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>toyota rav4 4</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,49 +905,49 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-rav4-4-2013-2018/navigatie-dedicata-cu-android-toyota-rav4-iv-2013-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -957,19 +957,19 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -981,12 +981,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ford mondeo 3</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2000-2007</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -994,12 +994,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ford mondeo 3</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2000-2007</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1009,36 +1009,36 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-3-2000-2007/navigatie-dedicata-cu-android-ford-mondeo-iii-2000-2007-clima-automata-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>kia sorento</t>
+          <t>ford mondeo 3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2013-2015</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1046,12 +1046,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>kia sorento 2</t>
+          <t>ford mondeo 3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1073,24 +1073,24 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-3-2000-2007/navigatie-dedicata-cu-android-ford-mondeo-iii-2000-2007-clima-automata-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>mazda</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>mazda 3</t>
+          <t>kia sorento</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2013-2015</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>mazda 3</t>
+          <t>kia sorento 2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2013-2019</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1113,36 +1113,36 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>mazda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2004-2010</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>opel astra h</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2013-2019</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1165,36 +1165,36 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>afisaj/comenzi clima</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>toyota avensis t27</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2004-2010</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1202,12 +1202,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>toyota avensis t27</t>
+          <t>opel astra h</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1217,49 +1217,49 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Aerul conditionat va putea fi controlat in continuare din butoanele fizice ale masinii, insa informatiile despre climatizare nu vor fi afisate pe ecranul navigatiei.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>afisaj/comenzi clima</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-astra-h-2004-2014/navigatie-dedicata-cu-android-opel-astra-h-2004-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi-2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>audi</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>audi a4 b8</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2007-2017</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1269,36 +1269,36 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>audi</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ford kuga</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ford kuga 1</t>
+          <t>audi a4 b8</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2007-2017</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat si mufa AUX in. Nu se poate monta pe masini dotate cu Audi CD Changer.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1333,37 +1333,37 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-audi-a4-b8-2007-2017/interfata-audio-video-cu-android-auto-si-carplay-audi-a4-b8-a5-8t-2007-2017-cu-navigatie-mmi-2g</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>ford kuga 1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Daca masina are navigatie originala Blaupunkt este necesar un modul control aer conditionat care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1385,24 +1385,24 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-kuga-1-2008-2012/navigatie-dedicata-cu-android-ford-kuga-i-2008-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2011-2017</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1410,12 +1410,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ford mondeo 4</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2007-2014</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1425,49 +1425,49 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>citroen</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>citroen c4 aircross</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2012-2017</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>citroen c4 aircross</t>
+          <t>ford mondeo 4</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2012-2017</t>
+          <t>2007-2014</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1477,19 +1477,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica. Daca masina nu are plus contact in mufa de alimentare a aparatului radio original este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-aircross-2012-2017/navigatie-dedicata-cu-android-citroen-c4-aircross-2012-2017-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-4-2007-2014/navigatie-dedicata-cu-android-ford-mondeo-iv-2007-2014-negru-2gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1501,12 +1501,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>citroen c4</t>
+          <t>citroen c4 aircross</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1548,17 +1548,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>citroen</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>dupa 2021</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>citroen c4 aircross</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1581,19 +1581,19 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-aircross-2012-2017/navigatie-dedicata-cu-android-citroen-c4-aircross-2012-2017-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen</t>
         </is>
       </c>
     </row>
@@ -1605,12 +1605,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>dupa 2013</t>
+          <t>dupa 2021</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1652,17 +1652,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>honda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>honda crv</t>
+          <t>ford transit connect</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>dupa 2013</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>honda cr v 3</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1685,19 +1685,19 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1722,12 +1722,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>honda cr v 4</t>
+          <t>honda cr v 3</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2012-2018</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1737,36 +1737,36 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-3-2006-2012/navigatie-dedicata-cu-android-honda-cr-v-iii-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>hyundai</t>
+          <t>honda</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>honda crv</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>hyundai ix35</t>
+          <t>honda cr v 4</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2012-2018</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1789,36 +1789,36 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are navigatie originala este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-honda-cr-v-4-2012-2018/navigatie-dedicata-cu-android-honda-cr-v-iv-2012-2018-6gb-ram-radio-gps-dual-zone-display-hd-qled-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>hyundai</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>kia sportage</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>kia sportage 3</t>
+          <t>hyundai ix35</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1853,24 +1853,24 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-hyundai-ix35-2009-2015/navigatie-dedicata-cu-android-hyundai-ix35-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>mitsubishi</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2010-2016</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>kia sportage 3</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>dupa 2010</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1905,24 +1905,24 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-3-2010-2016/navigatie-dedicata-cu-android-kia-sportage-2010-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>opel insignia</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2008-2013</t>
+          <t>2010-2016</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>opel insignia a</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2008-2017</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1945,19 +1945,19 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2013-2017</t>
+          <t>2008-2013</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -2016,30 +2016,30 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>mercedes benz c class w203</t>
+          <t>opel insignia</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2000-2004</t>
+          <t>2013-2017</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mercedes c class w203</t>
+          <t>opel insignia a</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2000-2007</t>
+          <t>2008-2017</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are sistemul audio pe fibra optica (are amplificator sau magazie de cd-uri) este necesar un cablu suplimentar de 6m care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au din fabrica sistem de sunet Infinity.</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-c-class-w203-2000-2007/navigatie-dedicata-cu-android-mercedes-c-class-w203-2000-2004-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-insignia-a-2008-2017/navigatie-dedicata-cu-android-opel-insignia-a-2008-2013-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2004-2007</t>
+          <t>2000-2004</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2120,30 +2120,30 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mercedes benz c class w203</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2014-2020</t>
+          <t>2004-2007</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mercedes c class w203</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2153,36 +2153,36 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are sistemul audio pe fibra optica (are amplificator sau magazie de cd-uri) este necesar un cablu suplimentar de 6m care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-c-class-w203-2000-2007/navigatie-dedicata-cu-android-mercedes-c-class-w203-2000-2004-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>kia</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>kia sorento</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2009-2012</t>
+          <t>2014-2020</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2190,12 +2190,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>kia sorento 2</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2205,19 +2205,19 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2229,12 +2229,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>kia sportage</t>
+          <t>kia sorento</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2009-2012</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2242,12 +2242,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>kia sportage 4</t>
+          <t>kia sorento 2</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2016-2021</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2257,19 +2257,19 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-4-2016-2021/navigatie-dedicata-cu-android-kia-sportage-2016-2018-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sorento-2-2009-2015/navigatie-dedicata-cu-android-kia-sorento-2012-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2018-2019</t>
+          <t>2016-2018</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2018-2019</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2380,17 +2380,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>mazda</t>
+          <t>kia</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>mazda cx 3</t>
+          <t>kia sportage</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2014-2021</t>
+          <t>2019-2021</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2398,12 +2398,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mazda 3</t>
+          <t>kia sportage 4</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2013-2019</t>
+          <t>2016-2021</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2413,36 +2413,36 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-kia-sportage-4-2016-2021/navigatie-dedicata-cu-android-kia-sportage-2016-2018-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>mitsubishi</t>
+          <t>mazda</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>mazda cx 3</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2014-2021</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2450,12 +2450,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>mitsubishi asx</t>
+          <t>mazda 3</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dupa 2010</t>
+          <t>2013-2019</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2465,19 +2465,19 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat. Navigatia este compatibila si cu masinile cu sistem audio Bose.</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>sistem audio amplificat din fabrica</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mazda-3-2013-2019/navigatie-dedicata-cu-android-mazda-3-2013-2019-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2017-2019</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2536,17 +2536,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>mitsubishi</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>toyota avensis</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2015-2018</t>
+          <t>2020-2022</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2554,12 +2554,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>toyota avensis t27</t>
+          <t>mitsubishi asx</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>dupa 2010</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
+          <t>Daca masina are amplificator Rockford este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2581,24 +2581,24 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mitsubishi-asx-dupa-2010/navigatie-dedicata-cu-android-mitsubishi-asx-dupa-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>toyota avensis</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2019-2024</t>
+          <t>2015-2018</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2606,12 +2606,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>vw transporter t6</t>
+          <t>toyota avensis t27</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2621,49 +2621,49 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>sistem audio amplificat din fabrica</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-avensis-t27-2009-2018/navigatie-dedicata-cu-android-toyota-avensis-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ford mondeo</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2000-2007</t>
+          <t>2019-2024</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ford mondeo 3</t>
+          <t>vw transporter t6</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2000-2007</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2673,19 +2673,19 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are rotile de reglare sub grilele de ventilatie, acestea vor trebui scoase pentru a putea monta navigatia.</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-3-2000-2007/navigatie-dedicata-cu-android-ford-mondeo-iii-2000-2007-clima-automata-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t6-dupa-2015/navigatie-dedicata-cu-android-vw-transporter-caravelle-multivan-t6-2015-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
@@ -2697,25 +2697,25 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>ford mondeo</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ford focus 3</t>
+          <t>ford mondeo 3</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2011-2018</t>
+          <t>2000-2007</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2725,19 +2725,19 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-mondeo-3-2000-2007/navigatie-dedicata-cu-android-ford-mondeo-iii-2000-2007-clima-automata-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5</t>
         </is>
       </c>
     </row>
@@ -2749,12 +2749,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ford transit courier</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2014-2018</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>ford focus 3</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>dupa 2014</t>
+          <t>2011-2018</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
+          <t>Daca masina are 12 senzori de parcare originali (6 fata si 6 spate), acestia vor fi preluati de navigatie doar vizual, nu si acustic.</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2789,37 +2789,37 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-3-2011-2018/navigatie-dedicata-cu-android-ford-focus-iii-2011-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>bmw x1 e84 cic</t>
+          <t>ford transit courier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>2014-2018</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>bmw x1 e84</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2009-2015</t>
+          <t>dupa 2014</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2829,19 +2829,19 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
+          <t>Daca masina are ecran pe bord care afiseaza data si ora, dupa montaj va ramane un mic spatiu gol in spatele navigatiei.</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-dupa-2014/navigatie-dedicata-cu-android-ford-transit-2014-2020-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -2853,12 +2853,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>bmw x3 f25 cic</t>
+          <t>bmw x1 e84 cic</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2011-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2866,12 +2866,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>bmw x3 f25</t>
+          <t>bmw x1 e84</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2010-2017</t>
+          <t>2009-2015</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2881,19 +2881,19 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
+          <t>Nu se poate monta pe masini care au navigatie originala din fabrica.</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>altceva — de citit</t>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x1-e84-2009-2015/navigatie-dedicata-cu-android-bmw-x1-e84-2009-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>bmw x3 f25 nbt</t>
+          <t>bmw x3 f25 cic</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2952,26 +2952,30 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NISSAN</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>(niciun model potrivit in catalogul nostru)</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>bmw x3 f25 nbt</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2011-2017</t>
+        </is>
+      </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>nissan qashqai 1</t>
+          <t>bmw x3 f25</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2010-2017</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2981,26 +2985,26 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
+          <t>Pentru a putea fi montata interfata, masina trebuie sa aiba AUX activat. In cazul masinilor cu camere 360 din fabrica, acestea vor fi afisate, dar nu va fi posibila schimbarea modului de vizualizare.</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>cere cablu/adaptor separat</t>
+          <t>altceva — de citit</t>
         </is>
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-bmw-x3-f25-2010-2017/interfata-audio-video-cu-android-auto-si-carplay-bmw-x3-f25-cu-navigatie-nbt-nbt-evo-id4-2013-2016</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>NISSAN</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3014,12 +3018,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>toyota corolla e18</t>
+          <t>nissan qashqai 1</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2013-2018</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3029,93 +3033,97 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+          <t>Daca masina are navigatie originala sau camera de marsarier este necesar un cablu suplimentar care se achizitioneaza separat.</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+          <t>cere cablu/adaptor separat</t>
         </is>
       </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-nissan-qashqai-1-2006-2014/navigatie-dedicata-cu-android-nissan-qashqai-i-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-7-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>vw tiguan</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>2007-2016</t>
-        </is>
-      </c>
+          <t>(niciun model potrivit in catalogul nostru)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>vw tiguan 1</t>
+          <t>toyota corolla e18</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2007-2018</t>
+          <t>2013-2018</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr"/>
-      <c r="I51" s="2" t="inlineStr"/>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Daca masina are amplificator sau navigatie originala si camera de marsarier este nevoie de un cablu adaptor care se achizitioneaza separat. Nu se poate monta pe masini cu butonul de avarii patrat. Pentru a putea fi montata, este necesar sa se decupeze o portiune mica de plastic din interiorul bordului.</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>incompatibilitate cu navigatia de fabrica (PROBABIL limitarea LOR, nu a masinii)</t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e18-2013-2018/navigatie-dedicata-cu-android-toyota-corolla-2017-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ford focus</t>
+          <t>vw tiguan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2007-2016</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>vw tiguan 1</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2007-2018</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3129,37 +3137,37 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-tiguan-1-2007-2018/navigatie-dedicata-cu-android-vw-tiguan-i-2007-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3173,7 +3181,7 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
@@ -3185,12 +3193,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3198,12 +3206,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>vw scirocco</t>
+          <t>vw golf 5</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2008-2018</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3217,37 +3225,37 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>skoda octavia</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>skoda octavia 2</t>
+          <t>vw scirocco</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2008-2018</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3261,24 +3269,24 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-scirocco-2008-2018/navigatie-dedicata-cu-android-vw-scirocco-2008-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>vw jetta</t>
+          <t>skoda octavia</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2006-2010</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3286,12 +3294,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>vw jetta 3</t>
+          <t>skoda octavia 2</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3305,7 +3313,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-octavia-2-2004-2013/navigatie-dedicata-cu-android-skoda-octavia-ii-2004-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
         </is>
       </c>
     </row>
@@ -3317,12 +3325,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>vw passat b6</t>
+          <t>vw jetta</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2005-2010</t>
+          <t>2006-2010</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3330,12 +3338,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>vw jetta 3</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3349,7 +3357,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-jetta-3-2004-2011/navigatie-dedicata-cu-android-vw-jetta-iii-2004-2011-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -3361,12 +3369,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw passat b6</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2005-2010</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3374,12 +3382,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>vw polo 6r</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3393,7 +3401,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -3405,12 +3413,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>vw touran</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2003-2013</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3418,12 +3426,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>vw touran 1</t>
+          <t>vw polo 6r</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3437,7 +3445,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-6r-2009-2018/navigatie-dedicata-cu-android-vw-polo-6r-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -3462,12 +3470,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>vw touran 2</t>
+          <t>vw touran 1</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3481,7 +3489,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-2-2010-2015/navigatie-dedicata-cu-android-vw-touran-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-1-2003-2010/navigatie-dedicata-cu-android-vw-touran-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -3493,25 +3501,25 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>vw polo</t>
+          <t>vw touran</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2001-2009</t>
+          <t>2003-2013</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>vw polo 9n</t>
+          <t>vw touran 2</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2001-2012</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3525,37 +3533,37 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-9n-2001-2012/navigatie-dedicata-cu-android-vw-polo-9n-2001-2012-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-touran-2-2010-2015/navigatie-dedicata-cu-android-vw-touran-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw polo</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2015-2022</t>
+          <t>2001-2009</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw polo 9n</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>dupa 2015</t>
+          <t>2001-2012</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3569,24 +3577,24 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-polo-9n-2001-2012/navigatie-dedicata-cu-android-vw-polo-9n-2001-2012-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>mercedes benz vito 3</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2012-2021</t>
+          <t>2015-2022</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3594,12 +3602,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>dupa 2015</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3613,37 +3621,37 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-dupa-2015/navigatie-dedicata-cu-android-ford-ranger-dupa-2015-cu-navigatie-originala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>opel</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>opel zafira</t>
+          <t>mercedes benz vito 3</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2012-2021</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>opel zafira b</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3657,37 +3665,37 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>opel</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>vw passat b7</t>
+          <t>opel zafira</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>vw passat b6 b7</t>
+          <t>opel zafira b</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2005-2015</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3701,37 +3709,37 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-opel-zafira-b-2005-2014/navigatie-dedicata-cu-android-opel-zafira-b-2005-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b7</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2007-2015</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>vw passat b6 b7</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2005-2015</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3745,24 +3753,24 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-passat-b6-b7-2005-2015/navigatie-dedicata-cu-android-vw-passat-b6-b7-2005-2015-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ford fiesta</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2007-2015</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3770,12 +3778,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ford fiesta 5</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2002-2008</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3789,24 +3797,24 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>mercedes benz viano</t>
+          <t>ford fiesta</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3814,12 +3822,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>ford fiesta 5</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2002-2008</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3833,7 +3841,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-fiesta-5-2002-2008/navigatie-dedicata-cu-android-ford-fiesta-v-2005-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -3845,12 +3853,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>mercedes benz vito</t>
+          <t>mercedes benz viano</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2003-2012</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3858,12 +3866,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3877,24 +3885,24 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>mercedes benz vito</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2003-2012</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3902,12 +3910,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3921,7 +3929,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -3933,12 +3941,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -3990,12 +3998,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>seat altea xl</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2006-2015</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -4009,7 +4017,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-2004-2015/navigatie-dedicata-cu-android-seat-altea-2004-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
@@ -4021,12 +4029,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>seat altea</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2004-2015</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4065,12 +4073,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>seat leon</t>
+          <t>seat altea</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2004-2015</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4078,12 +4086,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>seat leon 1p</t>
+          <t>seat altea xl</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2005-2013</t>
+          <t>2006-2015</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4097,24 +4105,24 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-altea-xl-2006-2015/navigatie-dedicata-cu-android-seat-altea-xl-2006-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>seat leon</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2012-2017</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4122,12 +4130,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>seat leon 1p</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2005-2013</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4141,24 +4149,24 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-leon-1p-2005-2013/navigatie-dedicata-cu-android-seat-leon-1p-2005-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>seat toledo</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2004-2009</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4166,12 +4174,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>seat toledo 3</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2004-2009</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -4185,24 +4193,24 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-toledo-3-2004-2009/navigatie-dedicata-cu-android-seat-toledo-iii-2004-2009-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>seat toledo iv</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2012-2019</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4210,12 +4218,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>seat toledo 4</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2012-2019</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -4229,24 +4237,24 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-seat-toledo-4-2012-2019/navigatie-dedicata-cu-android-seat-toledo-iv-2012-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>skoda fabia</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4254,12 +4262,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>skoda fabia 2</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4273,37 +4281,37 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-fabia-2-2006-2014/navigatie-dedicata-cu-android-skoda-fabia-ii-2006-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2010-2013</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>skoda rapid</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4317,37 +4325,37 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>skoda yeti</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2008-2012</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>skoda yeti</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4361,37 +4369,37 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-yeti-2009-2018/navigatie-dedicata-cu-android-skoda-yeti-2009-2018-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>vw golf plus</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2004-2014</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4405,37 +4413,37 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ford ranger f250</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4449,37 +4457,37 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>toyota auris e15</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2006-2012</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4493,37 +4501,37 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2005-2014</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4537,37 +4545,37 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2008-2012</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>vw multivan t5</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4581,37 +4589,37 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2003-2009</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>vw transporter t5</t>
+          <t>dacia logan 2</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2003-2015</t>
+          <t>2012-2020</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4625,37 +4633,37 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>citroen</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>citroen c4</t>
+          <t>ford ranger f250</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>citroen c4</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4669,37 +4677,37 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-2009-2018/navigatie-dedicata-cu-android-citroen-c4-ii-2009-2018-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-10</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>citroen</t>
+          <t>toyota</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>citroen c4 aircross</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2012-2017</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>citroen c4</t>
+          <t>toyota auris e15</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2009-2018</t>
+          <t>2006-2012</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4713,7 +4721,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-2009-2018/navigatie-dedicata-cu-android-citroen-c4-ii-2009-2018-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-10</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-auris-e15-2006-2012/navigatie-dedicata-cu-android-toyota-auris-2006-2012-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
@@ -4725,25 +4733,25 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2011-2016</t>
+          <t>2005-2014</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>ford ranger</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2011-2015</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4757,37 +4765,37 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>dacia duster</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2015-2020</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>dacia duster 1</t>
+          <t>vw multivan t5</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2010-2018</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4801,37 +4809,37 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-multivan-t5-2003-2015/navigatie-dedicata-cu-android-vw-multivan-v-2003-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>vw</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2003-2009</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>mercedes viano</t>
+          <t>vw transporter t5</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2003-2014</t>
+          <t>2003-2015</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4845,37 +4853,37 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-transporter-t5-2003-2015/navigatie-dedicata-cu-android-vw-transporter-t5-2010-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Mercedes Benz</t>
+          <t>citroen</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>mercedes benz vito viano w639</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2010-2015</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>mercedes vito</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>dupa 2003</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4889,37 +4897,37 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-2009-2018/navigatie-dedicata-cu-android-citroen-c4-ii-2009-2018-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-10</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>citroen</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>citroen c4 aircross</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2012-2017</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>ford focus 2</t>
+          <t>citroen c4</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2009-2018</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4933,37 +4941,37 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-citroen-c4-2009-2018/navigatie-dedicata-cu-android-citroen-c4-ii-2009-2018-clima-automata-1gb-ram-radio-gps-dual-zone-display-hd-ips-10</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2011-2016</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>dacia logan 1</t>
+          <t>ford ranger</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2004-2013</t>
+          <t>2011-2015</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4977,37 +4985,37 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-ranger-2011-2015/navigatie-dedicata-cu-android-ford-ranger-2011-2015-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>fiat</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>fiat 500 l</t>
+          <t>dacia duster</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>dupa 2012</t>
+          <t>2015-2020</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>fiat 500</t>
+          <t>dacia duster 1</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2007-2020</t>
+          <t>2010-2018</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -5021,37 +5029,37 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-duster-1-2010-2018/navigatie-dedicata-cu-android-dacia-duster-i-2013-2018-2gb-ram-radio-gps-dual-zone-display-hd-8-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ford transit connect</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2008-2011</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ford transit</t>
+          <t>mercedes viano</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2006-2014</t>
+          <t>2003-2014</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -5065,37 +5073,37 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-viano-2003-2014/navigatie-dedicata-cu-android-mercedes-viano-2007-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>Mercedes Benz</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>renault megane iii</t>
+          <t>mercedes benz vito viano w639</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>2010-2015</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>renault megane 3</t>
+          <t>mercedes vito</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2009-2016</t>
+          <t>dupa 2003</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -5109,37 +5117,37 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-mercedes-vito-dupa-2003/navigatie-dedicata-cu-android-mercedes-vito-dupa-2006-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>skoda rapid</t>
+          <t>ford focus 2</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -5153,24 +5161,24 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-focus-2-2004-2011/navigatie-dedicata-cu-android-ford-focus-ii-2004-2011-clima-manuala-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>toyota</t>
+          <t>dacia</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2004-2008</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5178,12 +5186,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>toyota corolla e15</t>
+          <t>dacia logan 1</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2007-2013</t>
+          <t>2004-2013</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -5197,24 +5205,24 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-1-2004-2013/navigatie-dedicata-cu-android-dacia-logan-i-2004-2008-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>fiat</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>fiat 500 l</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>dupa 2012</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5222,12 +5230,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>vw golf 5</t>
+          <t>fiat 500</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2003-2010</t>
+          <t>2007-2020</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -5241,24 +5249,24 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-fiat-500-2007-2020/navigatie-dedicata-cu-android-fiat-500-2015-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>vw</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>vw golf</t>
+          <t>ford transit connect</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2004-2008</t>
+          <t>2008-2011</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5266,12 +5274,12 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>vw golf plus</t>
+          <t>ford transit</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2004-2014</t>
+          <t>2006-2014</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -5285,37 +5293,37 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+          <t>https://www.navigatiiandroid.ro/navigatie-ford-transit-2006-2014/navigatie-dedicata-cu-android-ford-transit-2006-2014-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi-fi</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>dacia</t>
+          <t>renault</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>dacia logan</t>
+          <t>renault megane iii</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>dacia logan 2</t>
+          <t>renault megane 3</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2012-2020</t>
+          <t>2009-2016</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -5329,6 +5337,226 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-renault-megane-3-2009-2016/navigatie-dedicata-cu-android-renault-megane-iii-2009-2016-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>skoda</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2017-2019</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>9</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>skoda rapid</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2011-2019</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-skoda-rapid-2011-2019/navigatie-dedicata-cu-android-skoda-rapid-2011-2019-12gb-ram-radio-gps-dual-zone-display-2k-qled-9-5-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>toyota</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>9</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>toyota corolla e15</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>2007-2013</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-toyota-corolla-e15-2007-2013/navigatie-dedicata-cu-android-toyota-corolla-2007-2013-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>9</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>vw golf 5</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr"/>
+      <c r="I105" s="2" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-5-2003-2010/navigatie-dedicata-cu-android-vw-golf-v-2003-2010-1gb-ram-radio-gps-dual-zone-display-hd-ips-10-touchscreen-internet-wi-fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>vw</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>vw golf</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>2004-2008</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>9</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>vw golf plus</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>2004-2014</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>https://www.navigatiiandroid.ro/navigatie-vw-golf-plus-2004-2014/navigatie-dedicata-cu-android-vw-golf-plus-2004-2014-12gb-ram-radio-gps-dual-zone-display-2k-qled-10-36-touchscreen-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>dacia</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>dacia logan</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>3</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>dacia logan 2</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>2012-2020</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr"/>
+      <c r="I107" s="2" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
+        <is>
           <t>https://www.navigatiiandroid.ro/navigatie-dacia-logan-2-2012-2020/navigatie-dedicata-cu-android-dacia-logan-ii-2012-2020-1gb-ram-radio-gps-dual-zone-display-hd-ips-9-touchscreen-internet-wi</t>
         </is>
       </c>

</xml_diff>